<commit_message>
Added system token for pipeline validation
</commit_message>
<xml_diff>
--- a/datasets/2024_national_churches_trust_360_giving_data.xlsx
+++ b/datasets/2024_national_churches_trust_360_giving_data.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Mamiko\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Mamiko\Desktop\Github\national-church-trust-giving\datasets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{14269596-C95D-4AF1-B6B8-0189D38AA92F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C313B180-F8E7-408E-A4CC-B6F9842F7F51}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{01585C1E-420D-42BD-93F3-2E2BD389EEDC}"/>
+    <workbookView xWindow="32160" yWindow="3360" windowWidth="19425" windowHeight="10305" xr2:uid="{01585C1E-420D-42BD-93F3-2E2BD389EEDC}"/>
   </bookViews>
   <sheets>
     <sheet name="FINAL2024NationalChurchesTrust3" sheetId="1" r:id="rId1"/>
@@ -6010,11 +6010,11 @@
   <cols>
     <col min="1" max="1" width="24.90625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="24.6328125" customWidth="1"/>
-    <col min="3" max="3" width="30.1796875" customWidth="1"/>
+    <col min="3" max="3" width="21.7265625" customWidth="1"/>
     <col min="6" max="6" width="10.08984375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="16" customWidth="1"/>
-    <col min="9" max="9" width="13.54296875" customWidth="1"/>
-    <col min="10" max="10" width="11.36328125" customWidth="1"/>
+    <col min="8" max="8" width="19.453125" customWidth="1"/>
+    <col min="9" max="9" width="14.1796875" customWidth="1"/>
+    <col min="10" max="10" width="14.6328125" customWidth="1"/>
     <col min="18" max="18" width="20.453125" bestFit="1" customWidth="1"/>
     <col min="19" max="19" width="33.36328125" bestFit="1" customWidth="1"/>
     <col min="20" max="20" width="19.1796875" bestFit="1" customWidth="1"/>
@@ -24490,26 +24490,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<SharedContentType xmlns="Microsoft.SharePoint.Taxonomy.ContentTypeSync" SourceId="4d05856d-6385-46e0-852c-7b16b324f95d" ContentTypeId="0x0101004EC35B67BBCB2D44B550CAF14293968507" PreviousValue="false"/>
-</file>
-
-<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Grants" ma:contentTypeID="0x0101004EC35B67BBCB2D44B550CAF14293968507008D38BB02AF47354385C728769E668BED" ma:contentTypeVersion="5" ma:contentTypeDescription="for Grants library" ma:contentTypeScope="" ma:versionID="378d91f6995cc2109114b0098fc73cc5">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="c19ce98959e1c2270fec21953d0b7d94">
     <xsd:element name="properties">
@@ -24623,32 +24603,27 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6218C52E-082C-41AD-88C8-7BE1719AF0C7}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<SharedContentType xmlns="Microsoft.SharePoint.Taxonomy.ContentTypeSync" SourceId="4d05856d-6385-46e0-852c-7b16b324f95d" ContentTypeId="0x0101004EC35B67BBCB2D44B550CAF14293968507" PreviousValue="false"/>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B89E79BC-8A72-400B-88D9-E652CC976601}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D3803077-6984-4E5E-92EF-37369CD0A3E0}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="Microsoft.SharePoint.Taxonomy.ContentTypeSync"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{88A37213-8545-4D3B-99AD-AD419E16507E}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -24662,4 +24637,29 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D3803077-6984-4E5E-92EF-37369CD0A3E0}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="Microsoft.SharePoint.Taxonomy.ContentTypeSync"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B89E79BC-8A72-400B-88D9-E652CC976601}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6218C52E-082C-41AD-88C8-7BE1719AF0C7}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>